<commit_message>
B&N rev4 audit: resolve each difference from the drawings (v80j autonomy rule)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AxoFiJCtCJZAicZ6E1jrk
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/AUDITORIA_rev4/COMPARATIVA_AUDITORIA.xlsx
+++ b/cache_proyectos/barnes_noble/AUDITORIA_rev4/COMPARATIVA_AUDITORIA.xlsx
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every difference found by the auditor. The estimator decides; the take-off Excel was NOT changed. [DERIVED] = operation written; PENDING = not printed.</t>
+          <t>Every difference found by the auditor, resolved from the drawings (v80j total autonomy rule): the Recommendation column states which value is correct and why; what the plan does not resolve = RFI with delta and a conservative assumption. Take-off Excel NOT changed.</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Recommendation</t>
+          <t>Recommendation (correct value and why)</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Estimator to decide: add the two end-face finishes as type I rows (or note them inside C-H3a / C-H1-N). Framing LF does not change.</t>
+          <t>RESOLVED - correct: AUDITOR. 1/A-221 tags both end faces 'I SIM.'; I/A-221 gives the finish. Add type I end faces 1.21 LF: 5/8" FRT plywood 18.13 SF + GWB 12.08 SF (framing unchanged).</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Estimator decision RFI-18 (face-average arc) - observation only. If changed: type 4 = 82.68 LF.</t>
+          <t>RESOLVED - correct per plan: 25.20 LF centerline (printed 25'-1" on the face, 1/A-101). Take-off 25.68 is within 2 % and is estimator decision RFI-18 on record: keep take-off; no change.</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Move the two restroom ceilings to Type X W.R. (plan note is explicit).</t>
+          <t>RESOLVED - correct: AUDITOR. A-410 Partition Notes 2 is explicit (wall AND ceiling). Type X -120.2 SF, Type X W.R. +120.2 SF.</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Add as blocking (RFI-23 family) or confirm extent with an RFI.</t>
+          <t>RESOLVED - correct: AUDITOR (conservative). 11/A-200 prints the FR plywood area; extent not dimensioned -&gt; take the conservative upper bound 2.13 x 8'-0" = 17.0 SF 3/4" FRT plywood, RFI for exact extent (delta down to 0).</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Estimator decision - observation. The detail is printed; if in scope, add one row.</t>
+          <t>RFI (plan prints it, sizes do not). Conservative assumption: 2 pcs 3-5/8" stud backing x 4 ft = 8.0 LF + steel blocking 2 rows x 1.33 ft = 2.67 LF. Delta vs take-off: +8.0 LF stud, +2.67 LF blocking.</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Quantify from 3/A-221 (rule: do not ask what the plan resolves); keep only T.O. WD-1 as RFI.</t>
+          <t>RESOLVED - correct: AUDITOR. 3/A-221 + 6'-2" HOLD + A-121 7'-1" define the soffit. T.O. WD-1 not printed -&gt; RFI; conservative assumption: 5/8" FRT plywood full face 110.6 SF (delta if WD-1 lower: plywood -&gt; GWB 6.17 SF per ft).</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Estimator to decide whether the typical top-track detail applies (it is N.T.S. and generic).</t>
+          <t>RESOLVED - correct: AUDITOR (conservative). 8/A-410 is the typical top track detail and says 'TYP.'; it applies to every full-height wall with a ceiling on one face: +230.14 LF track (3-5/8" or 6" per wall). RFI only if the GC confirms it is not required.</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Cite the sheet of the note; if it does not exist, change the source text; if it does, add about 11.2 LF.</t>
+          <t>RFI. The quoted note was not found on A-410 / A-500 and the R.O. is not printed. Conservative assumption: +11.17 LF additional head track (doors 3 and 11). Fix the Material Summary citation (no sheet cited).</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Estimator decision - observation (RFI-11 scope).</t>
+          <t>RESOLVED - correct: AUDITOR (conservative). A-410 '*' note names KITCHEN and 2/A-410 names CAFE walls: Cafe Work Room GWB faces = Type X W.R. (up to 570 SF swap, total board unchanged).</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Add Corridor 110 wall tile to RFI-12; keep FRP under RFI-13.</t>
+          <t>RFI (A-510 gives the finish but not who installs FRP; A-002 lists wall tile as tenant / tenant contractor). Keep RFI-13 (FRP) and add Corridor 110 wall tile backer to RFI-12 with its delta.</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Estimator decision - observation.</t>
+          <t>RFI ('BY GC/FIXTURE INSTALLER' is ambiguous; W-3 count from A-111 not taken). Conservative assumption: carry the blocking strips per W-3 unit once the A-111 count is done; delta PENDING count.</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Estimator decision - observation: keep the exclusion visible in the bid clarifications.</t>
+          <t>RESOLVED - correct: TAKE-OFF. Insulation EXCLUDED is a skill standing rule (all projects); keep it in Clarifications.</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Add the stud breakdown (field / jambs / nodes / braces / posts) in 'Where it comes from'.</t>
+          <t>UNRESOLVED from the deliverables (one directed pass): both figures stay; take-off must show the stud breakdown (field / jambs / nodes / braces / posts).</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Same as above.</t>
+          <t>UNRESOLVED from the deliverables: both figures stay; add breakdown.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Add the face list for FRT plywood.</t>
+          <t>UNRESOLVED from the deliverables: both figures stay; add the FRT face list.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Update the two notes to the rev4 figures.</t>
+          <t>RESOLVED - correct: MATERIAL SUMMARY rev4 (15,579.48 / 1,020.33). Update ALC-07 / ALC-08 text.</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Confirm which count the estimator approved (31 vs 30 rows).</t>
+          <t>RESOLVED - correct: EXCEL 457.96 LF / 124 pcs (31 rows = ROUNDUP(38.833 x 12/16) + 1 at 16"); the decision record figure is outdated.</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Replace the internal file names with the plan citations.</t>
+          <t>RESOLVED - correct: cite N/SHEET in every row (format rule).</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Write the face heights in the Location / Status text of each row.</t>
+          <t>RESOLVED - correct: show per-face heights in each row (traceability rule).</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Update the notes.</t>
+          <t>RESOLVED - correct: update notes to 8/A-410 and to CLOSED RFI-15 / RFI-17; ALC-13 to RFI (or quantified per row 6).</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Rename (e.g. C-I-P.1) in Excel, markups and images together.</t>
+          <t>RESOLVED - correct: rename to C-I-P.1 in Excel, markups and images together.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Observation only.</t>
+          <t>RESOLVED - no change (template seal).</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Observation only.</t>
+          <t>RESOLVED - no change.</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Move the skill zips out of the project folder (manual, the service account cannot move).</t>
+          <t>RESOLVED - move the two skill zips out of the project folder (manual on Drive).</t>
         </is>
       </c>
     </row>

</xml_diff>